<commit_message>
Update ML4NLU Dot Product Excel file with new data
</commit_message>
<xml_diff>
--- a/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/01-ML4NLU-Dot-Product.xlsx
+++ b/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/01-ML4NLU-Dot-Product.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/peye9704_colorado_edu/Documents/2024/AIbyHand/spreadsheets/github/ai-by-hand-excel/workbook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hd/Desktop/Machine Learning/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61D2875F-AB07-7440-B7B6-333A2386914A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73C0BC3-3B14-0945-9E23-987CFA1624E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="18380" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" activeTab="4" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Exrcise 1-5" sheetId="1" r:id="rId1"/>
@@ -494,7 +494,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -604,6 +604,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -965,7 +968,7 @@
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="str">
         <f>IF(ISBLANK(E9)=TRUE,"NOT DONE",IF(B5=E9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -973,7 +976,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3" t="str">
         <f>IF(ISBLANK(H9)=TRUE,"NOT DONE",IF(G5=H9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1078,12 +1081,16 @@
       <c r="D9" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="23"/>
+      <c r="E9" s="23">
+        <v>15</v>
+      </c>
       <c r="F9" s="3"/>
       <c r="G9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="H9" s="24"/>
+      <c r="H9" s="24">
+        <v>3</v>
+      </c>
       <c r="I9" s="18" t="s">
         <v>49</v>
       </c>
@@ -1139,7 +1146,7 @@
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="str">
         <f>IF(ISBLANK(E19)=TRUE,"NOT DONE",IF(B15=E19,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -1147,7 +1154,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="str">
         <f>IF(ISBLANK(J17)=TRUE,"NOT DONE",IF(G15=J17,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -1219,7 +1226,9 @@
       <c r="G17" s="6"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="25"/>
+      <c r="J17" s="25">
+        <v>-3</v>
+      </c>
       <c r="K17" s="3"/>
     </row>
     <row r="18" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -1250,7 +1259,9 @@
       <c r="D19" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="25"/>
+      <c r="E19" s="25">
+        <v>8</v>
+      </c>
       <c r="F19" s="3"/>
       <c r="G19" s="9" t="s">
         <v>0</v>
@@ -1313,7 +1324,7 @@
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str">
         <f>IF(ISBLANK(E29)=TRUE,"NOT DONE",IF(B25=E29,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -1410,7 +1421,9 @@
       <c r="D29" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E29" s="25"/>
+      <c r="E29" s="25">
+        <v>-6</v>
+      </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
@@ -1482,11 +1495,11 @@
     <row r="3" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
         <f>IF(ISBLANK(F10)=TRUE,"NOT DONE",IF(B5=F10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="H3" t="str">
         <f>IF(ISBLANK(L10)=TRUE,"NOT DONE",IF(H5=L10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="19" x14ac:dyDescent="0.25">
@@ -1606,7 +1619,9 @@
       <c r="E10" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="23"/>
+      <c r="F10" s="23">
+        <v>3</v>
+      </c>
       <c r="G10" s="3"/>
       <c r="H10" s="9" t="s">
         <v>0</v>
@@ -1620,7 +1635,9 @@
       <c r="K10" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="L10" s="23"/>
+      <c r="L10" s="23">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" spans="1:15" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="10"/>
@@ -1668,7 +1685,7 @@
     <row r="14" spans="1:15" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="str">
         <f>IF(ISBLANK(F21)=TRUE,"NOT DONE",IF(B16=F21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1677,7 +1694,7 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="str">
         <f>IF(ISBLANK(L21)=TRUE,"NOT DONE",IF(H16=L21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -1799,7 +1816,9 @@
       <c r="E21" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="23"/>
+      <c r="F21" s="23">
+        <v>5</v>
+      </c>
       <c r="G21" s="3"/>
       <c r="H21" s="9" t="s">
         <v>0</v>
@@ -1813,7 +1832,9 @@
       <c r="K21" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="L21" s="23"/>
+      <c r="L21" s="23">
+        <v>-1</v>
+      </c>
     </row>
     <row r="22" spans="2:12" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="10"/>
@@ -1861,7 +1882,7 @@
     <row r="25" spans="2:12" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="str">
         <f>IF(ISBLANK(F32)=TRUE,"NOT DONE",IF(B27=F32,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1978,7 +1999,9 @@
       <c r="E32" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F32" s="23"/>
+      <c r="F32" s="23">
+        <v>7</v>
+      </c>
     </row>
     <row r="33" spans="2:6" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="10"/>
@@ -2033,11 +2056,11 @@
     <row r="3" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
         <f>IF(ISBLANK(F10)=TRUE,"NOT DONE",IF(B5=F10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="H3" t="str">
         <f>IF(ISBLANK(J10)=TRUE,"NOT DONE",IF(H5=J10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>INCORRECT</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -2151,14 +2174,18 @@
       <c r="E10" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="37">
+        <v>-6</v>
+      </c>
       <c r="H10" s="9" t="s">
         <v>0</v>
       </c>
       <c r="I10" s="28">
         <v>1</v>
       </c>
-      <c r="J10" s="35"/>
+      <c r="J10" s="35">
+        <v>0</v>
+      </c>
       <c r="K10" s="18" t="s">
         <v>49</v>
       </c>
@@ -2185,11 +2212,11 @@
     <row r="14" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f>IF(ISBLANK(F21)=TRUE,"NOT DONE",IF(B16=F21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="H14" t="str">
         <f>IF(ISBLANK(J21)=TRUE,"NOT DONE",IF(H16=J21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -2303,14 +2330,18 @@
       <c r="E21" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="23"/>
+      <c r="F21" s="23">
+        <v>0</v>
+      </c>
       <c r="H21" s="9" t="s">
         <v>0</v>
       </c>
       <c r="I21" s="28">
         <v>1</v>
       </c>
-      <c r="J21" s="35"/>
+      <c r="J21" s="35">
+        <v>-1</v>
+      </c>
       <c r="K21" s="18" t="s">
         <v>49</v>
       </c>
@@ -2337,7 +2368,7 @@
     <row r="25" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" t="str">
         <f>IF(ISBLANK(D32)=TRUE,"NOT DONE",IF(B27=D32,"CORRECT","INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="26" spans="2:12" ht="19" x14ac:dyDescent="0.25">
@@ -2402,7 +2433,9 @@
       <c r="C32" s="28">
         <v>1</v>
       </c>
-      <c r="D32" s="35"/>
+      <c r="D32" s="35">
+        <v>1</v>
+      </c>
       <c r="E32" s="18" t="s">
         <v>49</v>
       </c>
@@ -2460,11 +2493,11 @@
     <row r="3" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C3" t="str">
         <f>IF(ISBLANK(E10)=TRUE,"NOT DONE",IF(C5=E10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I3" t="str">
         <f>IF(ISBLANK(N11)=TRUE,"NOT DONE",IF(I5=N11,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -2578,7 +2611,9 @@
       <c r="D10" s="28">
         <v>1</v>
       </c>
-      <c r="E10" s="35"/>
+      <c r="E10" s="35">
+        <v>2</v>
+      </c>
       <c r="F10" s="18" t="s">
         <v>49</v>
       </c>
@@ -2617,7 +2652,9 @@
       <c r="M11" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="N11" s="23"/>
+      <c r="N11" s="23">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:14" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I12" s="5"/>
@@ -2632,11 +2669,11 @@
     <row r="14" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f>IF(ISBLANK(G22)=TRUE,"NOT DONE",IF(B16=G22,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I14" t="str">
         <f>IF(ISBLANK(L22)=TRUE,"NOT DONE",IF(I16=L22,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -2783,7 +2820,9 @@
       <c r="F22" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="G22" s="23"/>
+      <c r="G22" s="23">
+        <v>6</v>
+      </c>
       <c r="I22" s="9" t="s">
         <v>0</v>
       </c>
@@ -2793,7 +2832,9 @@
       <c r="K22" s="31">
         <v>0</v>
       </c>
-      <c r="L22" s="35"/>
+      <c r="L22" s="35">
+        <v>-1</v>
+      </c>
       <c r="M22" s="18" t="s">
         <v>49</v>
       </c>
@@ -2822,7 +2863,7 @@
     <row r="26" spans="2:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f>IF(ISBLANK(G34)=TRUE,"NOT DONE",IF(B28=G34,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="27" spans="2:14" ht="19" x14ac:dyDescent="0.25">
@@ -2912,7 +2953,9 @@
       <c r="F34" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="G34" s="23"/>
+      <c r="G34" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="35" spans="2:7" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="5"/>
@@ -2966,11 +3009,11 @@
     <row r="3" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
         <f>IF(ISBLANK(C11)=TRUE,"NOT DONE",IF(B5=C11,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>INCORRECT</v>
       </c>
       <c r="I3" t="str">
         <f>IF(ISBLANK(N9)=TRUE,"NOT DONE",IF(I5=N9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -3079,7 +3122,9 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="23"/>
+      <c r="N9" s="23">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:14" ht="19" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
@@ -3103,7 +3148,9 @@
       <c r="B11" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="39"/>
+      <c r="C11" s="45">
+        <v>1</v>
+      </c>
       <c r="D11" s="28">
         <v>1</v>
       </c>
@@ -3156,11 +3203,11 @@
     <row r="15" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f>IF(ISBLANK(C23)=TRUE,"NOT DONE",IF(B17=C23,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I15" t="str">
         <f>IF(ISBLANK(K23)=TRUE,"NOT DONE",IF(I17=K23,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -3295,7 +3342,9 @@
       <c r="B23" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="39"/>
+      <c r="C23" s="39">
+        <v>-1</v>
+      </c>
       <c r="D23" s="28">
         <v>1</v>
       </c>
@@ -3314,7 +3363,9 @@
       <c r="J23" s="28">
         <v>2</v>
       </c>
-      <c r="K23" s="35"/>
+      <c r="K23" s="35">
+        <v>-1</v>
+      </c>
       <c r="L23" s="29">
         <v>-9</v>
       </c>
@@ -3346,7 +3397,7 @@
     <row r="27" spans="2:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <f>IF(ISBLANK(G33)=TRUE,"NOT DONE",IF(B29=G33,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="28" spans="2:14" ht="19" x14ac:dyDescent="0.25">
@@ -3406,7 +3457,9 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
-      <c r="G33" s="23"/>
+      <c r="G33" s="23">
+        <v>-1</v>
+      </c>
     </row>
     <row r="34" spans="2:7" ht="19" x14ac:dyDescent="0.25">
       <c r="B34" s="4"/>

</xml_diff>